<commit_message>
No size limits, and faster on any document with the same minutes
No limits (a client's 290-page document was refused): MAX_SOURCE_CHARS, MAX_DOC_MB and
OCR_MAX_PAGES default to 0 = none (pages past 200 were skipped silently). The decisions, actions
and figures reads split a text too long for one model call into overlapping parts; the merge of a
long meeting reads as much as the model can; up to 50 ITEMs; a very large MoM can be re-prompted.

Faster (t5 took ~20 min): LLM_CONCURRENCY 2 -> 8 under one pod-wide gate; the main read's chunks
side by side; the windows and whole-file reads start beside the main read and are merged in the
same order; scanned pages OCR'd 4 at a time in page order (pod asks for 2 CPUs); an identical
request already running is joined, not redone. Old and new pipelines give identical minutes on
five documents with a deterministic stand-in model. 163 offline checks in tests/.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deploy/Service_Onboarding_Form_mom-prompt-service.xlsx
+++ b/deploy/Service_Onboarding_Form_mom-prompt-service.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="11" min="1" max="1"/>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="F46" s="13" t="inlineStr">
         <is>
-          <t>Parallel LLM calls per job</t>
+          <t>Model calls in flight at once for the pod; IBM allows 8 requests a second</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="F53" s="13" t="inlineStr">
         <is>
-          <t>Most scanned pages read per document, about 1 s each</t>
+          <t>Most scanned pages read per document; 0 = every page (a number skips the pages after it)</t>
         </is>
       </c>
     </row>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B54" s="13" t="inlineStr">
         <is>
-          <t>MIN_PAGE_TEXT_CHARS</t>
+          <t>OCR_WORKERS</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
@@ -1894,37 +1894,69 @@
       </c>
       <c r="F54" s="13" t="inlineStr">
         <is>
-          <t>A PDF page with less text of its own than this is OCR'd</t>
+          <t>Scanned pages read at the same time, one CPU core each (requests.cpu 2)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="13" t="inlineStr">
         <is>
+          <t>mom-prompt-service</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>MIN_PAGE_TEXT_CHARS</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F55" s="13" t="inlineStr">
+        <is>
+          <t>A PDF page with less text of its own than this is OCR'd</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="inlineStr">
+        <is>
           <t>all</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
+      <c r="B56" s="13" t="inlineStr">
         <is>
           <t>(other settings)</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
+      <c r="C56" s="13" t="inlineStr">
         <is>
           <t>Defaults in app/config.py and llama/config.py</t>
         </is>
       </c>
-      <c r="D55" s="13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E55" s="13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F55" s="13" t="inlineStr">
+      <c r="D56" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E56" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F56" s="13" t="inlineStr">
         <is>
           <t>Leave as shipped</t>
         </is>

</xml_diff>